<commit_message>
updated MIMIC preprocessing to be compatible with short term outcomes
</commit_message>
<xml_diff>
--- a/preprocessing/mimic_preprocessing/lab_preprocessing/selected_lab_values.xlsx
+++ b/preprocessing/mimic_preprocessing/lab_preprocessing/selected_lab_values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11113"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jk1/stroke_research/OPSUM/mimic_preprocessing/lab_preprocessing/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jk1/stroke_research/OPSUM/preprocessing/mimic_preprocessing/lab_preprocessing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A640DE2A-2E42-B943-86E7-D5F6B56FA526}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4A11EA3-8D2E-8245-A26C-8A655BB7CF08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="17920" windowHeight="21900" xr2:uid="{1804735D-6735-054A-9AAA-D63A2B9DDB72}"/>
+    <workbookView xWindow="17920" yWindow="600" windowWidth="17920" windowHeight="21800" xr2:uid="{1804735D-6735-054A-9AAA-D63A2B9DDB72}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="72">
   <si>
     <t>DPI_name</t>
   </si>
@@ -246,13 +246,19 @@
   </si>
   <si>
     <t>Urea Nitrogen</t>
+  </si>
+  <si>
+    <t>phosphates</t>
+  </si>
+  <si>
+    <t>Phosphate</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -282,6 +288,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF292929"/>
+      <name val="Menlo"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -303,11 +315,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -326,9 +339,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -366,7 +379,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -472,7 +485,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -614,7 +627,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -622,7 +635,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C429BBA-80F1-2045-BF64-7B1A2F6A9319}">
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.5" customWidth="1"/>
@@ -1046,6 +1059,23 @@
       </c>
       <c r="E27">
         <v>0.35709999999999997</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A28" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="D28">
+        <v>1</v>
+      </c>
+      <c r="E28">
+        <v>0.32290000000000002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated MIMIC preprocessing (#15)
* updated MIMIC preprocessing to be compatible with short term outcomes

* updated meta data processing for END

* updated imaging missingness computation and
table 1
</commit_message>
<xml_diff>
--- a/preprocessing/mimic_preprocessing/lab_preprocessing/selected_lab_values.xlsx
+++ b/preprocessing/mimic_preprocessing/lab_preprocessing/selected_lab_values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11113"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jk1/stroke_research/OPSUM/mimic_preprocessing/lab_preprocessing/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jk1/stroke_research/OPSUM/preprocessing/mimic_preprocessing/lab_preprocessing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A640DE2A-2E42-B943-86E7-D5F6B56FA526}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4A11EA3-8D2E-8245-A26C-8A655BB7CF08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="17920" windowHeight="21900" xr2:uid="{1804735D-6735-054A-9AAA-D63A2B9DDB72}"/>
+    <workbookView xWindow="17920" yWindow="600" windowWidth="17920" windowHeight="21800" xr2:uid="{1804735D-6735-054A-9AAA-D63A2B9DDB72}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="72">
   <si>
     <t>DPI_name</t>
   </si>
@@ -246,13 +246,19 @@
   </si>
   <si>
     <t>Urea Nitrogen</t>
+  </si>
+  <si>
+    <t>phosphates</t>
+  </si>
+  <si>
+    <t>Phosphate</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -282,6 +288,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF292929"/>
+      <name val="Menlo"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -303,11 +315,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -326,9 +339,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -366,7 +379,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -472,7 +485,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -614,7 +627,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -622,7 +635,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C429BBA-80F1-2045-BF64-7B1A2F6A9319}">
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.5" customWidth="1"/>
@@ -1046,6 +1059,23 @@
       </c>
       <c r="E27">
         <v>0.35709999999999997</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A28" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="D28">
+        <v>1</v>
+      </c>
+      <c r="E28">
+        <v>0.32290000000000002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>